<commit_message>
Add PEI and keep total indicators only
</commit_message>
<xml_diff>
--- a/data/processed/codebook.xlsx
+++ b/data/processed/codebook.xlsx
@@ -539,24 +539,24 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PDI</t>
+          <t>Programa investigador</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Official indicator PDI Total; official unit Personal.</t>
+          <t>Official PEI program dimension from PEI0301; blank for PDI/PTGAS rows.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PDI_ETC</t>
+          <t>PDI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Official indicator PDI en ETC; stored separately from PDI.</t>
+          <t>Official indicator PDI Total; official unit Personal.</t>
         </is>
       </c>
     </row>
@@ -575,12 +575,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PTGAS_ETC</t>
+          <t>PEI</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Official indicator PTGAS ETC; ETC note says Equivalente a tiempo completo.</t>
+          <t>Official PEI values from PEI0301; official unit Personal.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add student indicators dashboard data
</commit_message>
<xml_diff>
--- a/data/processed/codebook.xlsx
+++ b/data/processed/codebook.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,48 +539,96 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Programa investigador</t>
+          <t>Nivel académico</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Official PEI program dimension from PEI0301; blank for PDI/PTGAS rows.</t>
+          <t>Student level: Grado y ciclo, Máster or Doctorado.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PDI</t>
+          <t>Ámbito de estudio</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Official indicator PDI Total; official unit Personal.</t>
+          <t>Official student field dimension from SIIU ámbito de estudio tables.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PTGAS</t>
+          <t>Programa investigador</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Official indicator PTGAS Total; official unit Personal.</t>
+          <t>Official PEI program dimension from PEI0301; blank for PDI/PTGAS rows.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>PDI</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Official indicator PDI Total; official unit Personal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PTGAS</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Official indicator PTGAS Total; official unit Personal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>PEI</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Official PEI values from PEI0301; official unit Personal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Flujo</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Student flow: Estudiantes matriculados or Estudiantes egresados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Estudiantes</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Official student count; official unit Número de estudiantes.</t>
         </is>
       </c>
     </row>

</xml_diff>